<commit_message>
Combined scan results 2026-08-22
</commit_message>
<xml_diff>
--- a/results/2026-08-22.xlsx
+++ b/results/2026-08-22.xlsx
@@ -414,9 +414,895 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>1. 信號反轉-底背離</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2. 信號反轉-回升</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>3. 機會入場</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>4. 重新起漲</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>5. 空中加油</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ABUS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CDZI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ACRS</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ABSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CELC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AFRM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ACHV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ERIC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ALM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>IONS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ASND</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LBTYA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LOPE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ARGX</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>AXGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>QUBT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BIIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>AUPH</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CCEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CGAU</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CHRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CGON</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CLYM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CNR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CRON</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>COKE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CVSA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CSX</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CYRX</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DJCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>FCFS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>DUOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FRHC</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FANG</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FWONK</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GH</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>FOX</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>FROG</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>IBKR</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>GLNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>IDYA</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>GMAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>HALO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>IMMX</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>INBX</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>IMNM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>INCY</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>IMVT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MEDP</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>IRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MEOH</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>JAZZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MRX</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>KOPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>NDSN</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>KRNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LPTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>NWS</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MGTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PGEN</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PHVS</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PRLD</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SATL</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>RFAI</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SLDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TARS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>RZLT</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SBLK</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SHC</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SOPH</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SRRK</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SRTA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SSRM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>STOK</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>TRLV</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -427,9 +1313,586 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>強勢+站穩+大量</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>開漲+站穩</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>開漲+大量</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>開漲</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TMUS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>GDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ADPT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SOUN</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HTZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AMCR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ALM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BTU</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ASST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ARCC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CAKE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ARX</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CME</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AUGO</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CMCSA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EXE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BETA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BLSH</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DBX</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FBRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BSY</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BNTX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DFTX</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>IBKR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CGAU</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DXCM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CLBK</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CSX</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FIVN</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FUTU</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GEHC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MKTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>HALO</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DKNG</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NVAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EXLS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FIGR</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>FROG</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GH</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PURR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SBLK</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RVMD</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SBET</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SSRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>STRC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PPC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SHC</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>